<commit_message>
rm extra rownames from s4
</commit_message>
<xml_diff>
--- a/tables/results/TableS4.xlsx
+++ b/tables/results/TableS4.xlsx
@@ -40,25 +40,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">miRNA</t>
+          <t xml:space="preserve">miR-10b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">human_miRNA_id</t>
+          <t xml:space="preserve">hsa-miR-10b-5p</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mouse_miRNA_id</t>
+          <t xml:space="preserve">mmu-miR-10b-5p</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">class</t>
-        </is>
-      </c>
-      <c r="E2"/>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/17898713/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -68,12 +72,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-10b-5p</t>
+          <t xml:space="preserve">hsa-miR-10b-3p</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-10b-5p</t>
+          <t xml:space="preserve">mmu-miR-10b-3p</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -81,26 +85,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/17898713/</t>
-        </is>
-      </c>
+      <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-10b</t>
+          <t xml:space="preserve">miR-93</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-10b-3p</t>
+          <t xml:space="preserve">hsa-miR-93-5p</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-10b-3p</t>
+          <t xml:space="preserve">mmu-miR-93-5p</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -108,7 +108,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E4"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.nature.com/articles/srep23772</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -118,12 +122,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-93-5p</t>
+          <t xml:space="preserve">hsa-miR-93-3p</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-93-5p</t>
+          <t xml:space="preserve">mmu-miR-93-3p</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -131,26 +135,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.nature.com/articles/srep23772</t>
-        </is>
-      </c>
+      <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-93</t>
+          <t xml:space="preserve">miR-135b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-93-3p</t>
+          <t xml:space="preserve">hsa-miR-135b-3p</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-93-3p</t>
+          <t xml:space="preserve">mmu-miR-135b-3p</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -158,7 +158,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E6"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.nature.com/articles/ncomms2876</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -168,12 +172,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-135b-3p</t>
+          <t xml:space="preserve">hsa-miR-135b-5p</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-135b-3p</t>
+          <t xml:space="preserve">mmu-miR-135b-5p</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -181,26 +185,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.nature.com/articles/ncomms2876</t>
-        </is>
-      </c>
+      <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-135b</t>
+          <t xml:space="preserve">miR-183-5p</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-135b-5p</t>
+          <t xml:space="preserve">hsa-miR-183-5p</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-135b-5p</t>
+          <t xml:space="preserve">mmu-miR-183-5p</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -208,22 +208,26 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E8"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/30070321/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-183-5p</t>
+          <t xml:space="preserve">miR-208a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-183-5p</t>
+          <t xml:space="preserve">hsa-miR-208a-3p</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-183-5p</t>
+          <t xml:space="preserve">mmu-miR-208a-3p</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -233,7 +237,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/30070321/</t>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6755238/#:~:text=Herein%2C%20the%20results%20demonstrated%20that,for%20treating%20patients%20with%20NSCLC.</t>
         </is>
       </c>
     </row>
@@ -245,12 +249,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-208a-3p</t>
+          <t xml:space="preserve">hsa-miR-208a-5p</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-208a-3p</t>
+          <t xml:space="preserve">mmu-miR-208a-5p</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -258,26 +262,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6755238/#:~:text=Herein%2C%20the%20results%20demonstrated%20that,for%20treating%20patients%20with%20NSCLC.</t>
-        </is>
-      </c>
+      <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-208a</t>
+          <t xml:space="preserve">miR-221</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-208a-5p</t>
+          <t xml:space="preserve">hsa-miR-221-3p</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-208a-5p</t>
+          <t xml:space="preserve">mmu-miR-221-3p</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -285,7 +285,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E11"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -295,12 +299,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-221-3p</t>
+          <t xml:space="preserve">hsa-miR-221-5p</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-221-3p</t>
+          <t xml:space="preserve">mmu-miR-221-5p</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -308,26 +312,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
-        </is>
-      </c>
+      <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-221</t>
+          <t xml:space="preserve">miR-222</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-221-5p</t>
+          <t xml:space="preserve">hsa-miR-222-3p</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-221-5p</t>
+          <t xml:space="preserve">mmu-miR-222-3p</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -335,7 +335,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E13"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -345,12 +349,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-222-3p</t>
+          <t xml:space="preserve">hsa-miR-222-5p</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-222-3p</t>
+          <t xml:space="preserve">mmu-miR-222-5p</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -358,34 +362,30 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
-        </is>
-      </c>
+      <c r="E14"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-222</t>
+          <t xml:space="preserve">miR-372</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-222-5p</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mmu-miR-222-5p</t>
-        </is>
-      </c>
+          <t xml:space="preserve">hsa-miR-372-3p</t>
+        </is>
+      </c>
+      <c r="C15"/>
       <c r="D15" t="inlineStr">
         <is>
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E15"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3551676/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-372-3p</t>
+          <t xml:space="preserve">hsa-miR-372-5p</t>
         </is>
       </c>
       <c r="C16"/>
@@ -404,21 +404,17 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3551676/</t>
-        </is>
-      </c>
+      <c r="E16"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-372</t>
+          <t xml:space="preserve">miR-373</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-372-5p</t>
+          <t xml:space="preserve">hsa-miR-373-3p</t>
         </is>
       </c>
       <c r="C17"/>
@@ -427,7 +423,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E17"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.tandfonline.com/doi/pdf/10.2147/OTT.S205582</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -437,7 +437,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-373-3p</t>
+          <t xml:space="preserve">hsa-miR-373-5p</t>
         </is>
       </c>
       <c r="C18"/>
@@ -446,30 +446,34 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.tandfonline.com/doi/pdf/10.2147/OTT.S205582</t>
-        </is>
-      </c>
+      <c r="E18"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-373</t>
+          <t xml:space="preserve">miR-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-373-5p</t>
-        </is>
-      </c>
-      <c r="C19"/>
+          <t xml:space="preserve">hsa-miR-24-1-5p</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mmu-miR-24-1-5p</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E19"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -479,12 +483,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-24-1-5p</t>
+          <t xml:space="preserve">hsa-miR-24-2-5p</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-24-1-5p</t>
+          <t xml:space="preserve">mmu-miR-24-2-5p</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -492,11 +496,7 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
-        </is>
-      </c>
+      <c r="E20"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -506,12 +506,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-24-2-5p</t>
+          <t xml:space="preserve">hsa-miR-24-3p</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-24-2-5p</t>
+          <t xml:space="preserve">mmu-miR-24-3p</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -524,17 +524,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-24</t>
+          <t xml:space="preserve">miR-23</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-24-3p</t>
+          <t xml:space="preserve">hsa-miR-23a-5p</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-24-3p</t>
+          <t xml:space="preserve">mmu-miR-23a-5p</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -542,7 +542,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E22"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -552,12 +556,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-23a-5p</t>
+          <t xml:space="preserve">hsa-miR-23a-3p</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-23a-5p</t>
+          <t xml:space="preserve">mmu-miR-23a-3p</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -565,11 +569,7 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
-        </is>
-      </c>
+      <c r="E23"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-23a-3p</t>
+          <t xml:space="preserve">hsa-miR-23b-5p</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-23a-3p</t>
+          <t xml:space="preserve">mmu-miR-23b-5p</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-23b-5p</t>
+          <t xml:space="preserve">hsa-miR-23b-3p</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-23b-5p</t>
+          <t xml:space="preserve">mmu-miR-23b-3p</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -620,17 +620,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-23</t>
+          <t xml:space="preserve">miR-27</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-23b-3p</t>
+          <t xml:space="preserve">hsa-miR-27a-3p</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-23b-3p</t>
+          <t xml:space="preserve">mmu-miR-27a-3p</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -638,7 +638,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E26"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -648,12 +652,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-27a-3p</t>
+          <t xml:space="preserve">hsa-miR-27a-5p</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-27a-3p</t>
+          <t xml:space="preserve">mmu-miR-27a-5p</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -661,11 +665,7 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://link.springer.com/article/10.1007/s11011-024-01394-9</t>
-        </is>
-      </c>
+      <c r="E27"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-27a-5p</t>
+          <t xml:space="preserve">hsa-miR-27b-3p</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-27a-5p</t>
+          <t xml:space="preserve">mmu-miR-27b-3p</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-27b-3p</t>
+          <t xml:space="preserve">hsa-miR-27b-5p</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-27b-3p</t>
+          <t xml:space="preserve">mmu-miR-27b-5p</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -716,17 +716,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-27</t>
+          <t xml:space="preserve">miR-196b</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-27b-5p</t>
+          <t xml:space="preserve">hsa-miR-196b-5p</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-27b-5p</t>
+          <t xml:space="preserve">mmu-miR-196b-5p</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -734,7 +734,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E30"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/25233933/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -744,12 +748,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-196b-5p</t>
+          <t xml:space="preserve">hsa-miR-196b-3p</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-196b-5p</t>
+          <t xml:space="preserve">mmu-miR-196b-3p</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -757,26 +761,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/25233933/</t>
-        </is>
-      </c>
+      <c r="E31"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-196b</t>
+          <t xml:space="preserve">miR-127</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-196b-3p</t>
+          <t xml:space="preserve">hsa-miR-127-3p</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-196b-3p</t>
+          <t xml:space="preserve">mmu-miR-127-3p</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -784,7 +784,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E32"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.spandidos-publications.com/10.3892/or.2014.3055</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -794,12 +798,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-127-3p</t>
+          <t xml:space="preserve">hsa-miR-127-5p</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-127-3p</t>
+          <t xml:space="preserve">mmu-miR-127-5p</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -807,47 +811,47 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.spandidos-publications.com/10.3892/or.2014.3055</t>
-        </is>
-      </c>
+      <c r="E33"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-127</t>
+          <t xml:space="preserve">miR-197-3p</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-127-5p</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mmu-miR-127-5p</t>
-        </is>
-      </c>
+          <t xml:space="preserve">hsa-miR-197-3p</t>
+        </is>
+      </c>
+      <c r="C34"/>
       <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E34"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24488097/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-197-3p</t>
+          <t xml:space="preserve">miR-21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-197-3p</t>
-        </is>
-      </c>
-      <c r="C35"/>
+          <t xml:space="preserve">hsa-miR-21-3p</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mmu-miR-21a-3p</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">OncomiR</t>
@@ -855,7 +859,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24488097/</t>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/16024602/</t>
         </is>
       </c>
     </row>
@@ -867,12 +871,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-21-3p</t>
+          <t xml:space="preserve">hsa-miR-21-5p</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-21a-3p</t>
+          <t xml:space="preserve">mmu-miR-21a-5p</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -880,26 +884,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/16024602/</t>
-        </is>
-      </c>
+      <c r="E36"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-21</t>
+          <t xml:space="preserve">miR-155</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-21-5p</t>
+          <t xml:space="preserve">hsa-miR-155-5p</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-21a-5p</t>
+          <t xml:space="preserve">mmu-miR-155-3p</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -907,7 +907,11 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E37"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/20354188/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -917,12 +921,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-155-5p</t>
+          <t xml:space="preserve">hsa-miR-155-3p</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-155-3p</t>
+          <t xml:space="preserve">mmu-miR-155-5p</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -930,26 +934,22 @@
           <t xml:space="preserve">OncomiR</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/20354188/</t>
-        </is>
-      </c>
+      <c r="E38"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-155</t>
+          <t xml:space="preserve">miR-17-5p</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-155-3p</t>
+          <t xml:space="preserve">hsa-miR-17-5p</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-155-5p</t>
+          <t xml:space="preserve">mmu-miR-17-5p</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -962,17 +962,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-17-5p</t>
+          <t xml:space="preserve">miR-18a</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-17-5p</t>
+          <t xml:space="preserve">hsa-miR-18a-3p</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-17-5p</t>
+          <t xml:space="preserve">mmu-miR-18a-3p</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-18a-3p</t>
+          <t xml:space="preserve">hsa-miR-18a-5p</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-18a-3p</t>
+          <t xml:space="preserve">mmu-miR-18a-5p</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1008,17 +1008,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-18a</t>
+          <t xml:space="preserve">miR-19a</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-18a-5p</t>
+          <t xml:space="preserve">hsa-miR-19a-3p</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-18a-5p</t>
+          <t xml:space="preserve">mmu-miR-19a-3p</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1036,12 +1036,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-19a-3p</t>
+          <t xml:space="preserve">hsa-miR-19a-5p</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-19a-3p</t>
+          <t xml:space="preserve">mmu-miR-19a-5p</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1054,17 +1054,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-19a</t>
+          <t xml:space="preserve">miR-19b</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-19a-5p</t>
+          <t xml:space="preserve">hsa-miR-19b-3p</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-19a-5p</t>
+          <t xml:space="preserve">mmu-miR-19b-3p</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-19b-3p</t>
+          <t xml:space="preserve">hsa-miR-19b-1-5p</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-19b-3p</t>
+          <t xml:space="preserve">mmu-miR-19b-1-5p</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-19b-1-5p</t>
+          <t xml:space="preserve">hsa-miR-19b-2-5p</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-19b-1-5p</t>
+          <t xml:space="preserve">mmu-miR-19b-2-5p</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1123,17 +1123,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-19b</t>
+          <t xml:space="preserve">miR-20a</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-19b-2-5p</t>
+          <t xml:space="preserve">hsa-miR-20a-5p</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-19b-2-5p</t>
+          <t xml:space="preserve">mmu-miR-20a-5p</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1151,12 +1151,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-20a-5p</t>
+          <t xml:space="preserve">hsa-miR-20a-3p</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-20a-5p</t>
+          <t xml:space="preserve">mmu-miR-20a-3p</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1169,17 +1169,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-20a</t>
+          <t xml:space="preserve">miR-92</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-20a-3p</t>
+          <t xml:space="preserve">hsa-miR-92b-3p</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-20a-3p</t>
+          <t xml:space="preserve">mmu-miR-92a-3p</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-92b-3p</t>
+          <t xml:space="preserve">hsa-miR-92a-1-5p</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-92a-3p</t>
+          <t xml:space="preserve">mmu-miR-92a-2-5p</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1220,12 +1220,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-92a-1-5p</t>
+          <t xml:space="preserve">hsa-miR-92a-2-5p</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-92a-2-5p</t>
+          <t xml:space="preserve">mmu-miR-92b-3p</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-92a-2-5p</t>
+          <t xml:space="preserve">hsa-miR-92b-5p</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-92b-3p</t>
+          <t xml:space="preserve">mmu-miR-92a-1-5p</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1264,14 +1264,10 @@
           <t xml:space="preserve">miR-92</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hsa-miR-92b-5p</t>
-        </is>
-      </c>
+      <c r="B53"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-92a-1-5p</t>
+          <t xml:space="preserve">mmu-miR-92b-5p</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1284,21 +1280,29 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-92</t>
-        </is>
-      </c>
-      <c r="B54"/>
+          <t xml:space="preserve">miR-15a</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hsa-miR-15a-3p</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-92b-5p</t>
+          <t xml:space="preserve">mmu-miR-15a-3p</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">OncomiR</t>
-        </is>
-      </c>
-      <c r="E54"/>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC8979810/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1308,12 +1312,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-15a-3p</t>
+          <t xml:space="preserve">hsa-miR-15a-5p</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-15a-3p</t>
+          <t xml:space="preserve">mmu-miR-15a-5p</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1321,26 +1325,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC8979810/</t>
-        </is>
-      </c>
+      <c r="E55"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-15a</t>
+          <t xml:space="preserve">miR-16-1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-15a-5p</t>
+          <t xml:space="preserve">hsa-miR-16-1-3p</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-15a-5p</t>
+          <t xml:space="preserve">mmu-miR-16-1-3p</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1348,22 +1348,26 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E56"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5593589/</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-16-1</t>
+          <t xml:space="preserve">miR-34a</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-16-1-3p</t>
+          <t xml:space="preserve">hsa-miR-34a-3p</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-16-1-3p</t>
+          <t xml:space="preserve">mmu-miR-34a-3p</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1373,7 +1377,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5593589/</t>
+          <t xml:space="preserve">https://www.pnas.org/doi/10.1073/pnas.0707351104</t>
         </is>
       </c>
     </row>
@@ -1385,12 +1389,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34a-3p</t>
+          <t xml:space="preserve">hsa-miR-34a-5p</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34a-3p</t>
+          <t xml:space="preserve">mmu-miR-34a-5p</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1398,26 +1402,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.pnas.org/doi/10.1073/pnas.0707351104</t>
-        </is>
-      </c>
+      <c r="E58"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-34a</t>
+          <t xml:space="preserve">miR-34b</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34a-5p</t>
+          <t xml:space="preserve">hsa-miR-34b-3p</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34a-5p</t>
+          <t xml:space="preserve">mmu-miR-34b-3p</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1425,7 +1425,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E59"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/23314612/</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1435,12 +1439,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34b-3p</t>
+          <t xml:space="preserve">hsa-miR-34b-5p</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34b-3p</t>
+          <t xml:space="preserve">mmu-miR-34b-5p</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1448,26 +1452,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/23314612/</t>
-        </is>
-      </c>
+      <c r="E60"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-34b</t>
+          <t xml:space="preserve">miR-34c</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34b-5p</t>
+          <t xml:space="preserve">hsa-miR-34c-5p</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34b-5p</t>
+          <t xml:space="preserve">mmu-miR-34c-5p</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1475,7 +1475,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E61"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6647009/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1485,12 +1489,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34c-5p</t>
+          <t xml:space="preserve">hsa-miR-34c-3p</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34c-5p</t>
+          <t xml:space="preserve">mmu-miR-34c-3p</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1498,26 +1502,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6647009/</t>
-        </is>
-      </c>
+      <c r="E62"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-34c</t>
+          <t xml:space="preserve">miR-124</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-34c-3p</t>
+          <t xml:space="preserve">hsa-miR-124-3p</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-34c-3p</t>
+          <t xml:space="preserve">mmu-miR-124-3p</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1525,7 +1525,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E63"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC8198231/</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1535,12 +1539,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-124-3p</t>
+          <t xml:space="preserve">hsa-miR-124-5p</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-124-3p</t>
+          <t xml:space="preserve">mmu-miR-124-5p</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1548,26 +1552,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC8198231/</t>
-        </is>
-      </c>
+      <c r="E64"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-124</t>
+          <t xml:space="preserve">miR-125a</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-124-5p</t>
+          <t xml:space="preserve">hsa-miR-125a-5p</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-124-5p</t>
+          <t xml:space="preserve">mmu-miR-125a-5p</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1575,7 +1575,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E65"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4694830/</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1585,12 +1589,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-125a-5p</t>
+          <t xml:space="preserve">hsa-miR-125a-3p</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-125a-5p</t>
+          <t xml:space="preserve">mmu-miR-125a-3p</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1598,26 +1602,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4694830/</t>
-        </is>
-      </c>
+      <c r="E66"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-125a</t>
+          <t xml:space="preserve">miR-125b</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-125a-3p</t>
+          <t xml:space="preserve">hsa-miR-125b-5p</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-125a-3p</t>
+          <t xml:space="preserve">mmu-miR-125b-5p</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1625,7 +1625,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E67"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://aacrjournals.org/cancerres/article/71/10/3552/567653/miR-125b-Is-Methylated-and-Functions-as-a-Tumor</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1635,12 +1639,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-125b-5p</t>
+          <t xml:space="preserve">hsa-miR-125b-1-3p</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-125b-5p</t>
+          <t xml:space="preserve">mmu-miR-125b-2-3p</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1648,11 +1652,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://aacrjournals.org/cancerres/article/71/10/3552/567653/miR-125b-Is-Methylated-and-Functions-as-a-Tumor</t>
-        </is>
-      </c>
+      <c r="E68"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-125b-1-3p</t>
+          <t xml:space="preserve">hsa-miR-125b-2-3p</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-125b-2-3p</t>
+          <t xml:space="preserve">mmu-miR-125b-1-3p</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1680,17 +1680,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-125b</t>
+          <t xml:space="preserve">miR-143</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-125b-2-3p</t>
+          <t xml:space="preserve">hsa-miR-143-3p</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-125b-1-3p</t>
+          <t xml:space="preserve">mmu-miR-143-3p</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1698,7 +1698,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E70"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4170647/</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1708,12 +1712,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-143-3p</t>
+          <t xml:space="preserve">hsa-miR-143-5p</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-143-3p</t>
+          <t xml:space="preserve">mmu-miR-143-5p</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1721,26 +1725,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4170647/</t>
-        </is>
-      </c>
+      <c r="E71"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-143</t>
+          <t xml:space="preserve">miR-145</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-143-5p</t>
+          <t xml:space="preserve">hsa-miR-145-5p</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-143-5p</t>
+          <t xml:space="preserve">mmu-miR-145a-5p</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -1748,7 +1748,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E72"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6349084/</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1758,12 +1762,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-145-5p</t>
+          <t xml:space="preserve">hsa-miR-145-3p</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-145a-5p</t>
+          <t xml:space="preserve">mmu-miR-145-3p</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -1771,26 +1775,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6349084/</t>
-        </is>
-      </c>
+      <c r="E73"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-145</t>
+          <t xml:space="preserve">let-7a</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-145-3p</t>
+          <t xml:space="preserve">hsa-let-7a-5p</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-145-3p</t>
+          <t xml:space="preserve">mmu-let-7a-5p</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -1798,7 +1798,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E74"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/19787239/</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1808,12 +1812,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7a-5p</t>
+          <t xml:space="preserve">hsa-let-7a-3p</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7a-5p</t>
+          <t xml:space="preserve">mmu-let-7a-1-3p</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -1821,11 +1825,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/19787239/</t>
-        </is>
-      </c>
+      <c r="E75"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1835,12 +1835,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7a-3p</t>
+          <t xml:space="preserve">hsa-let-7a-2-3p</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7a-1-3p</t>
+          <t xml:space="preserve">mmu-let-7a-2-3p</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -1853,17 +1853,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">let-7a</t>
+          <t xml:space="preserve">let-7b</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7a-2-3p</t>
+          <t xml:space="preserve">hsa-let-7b-5p</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7a-2-3p</t>
+          <t xml:space="preserve">mmu-let-7b-5p</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -1871,7 +1871,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E77"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6341898/</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1881,12 +1885,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7b-5p</t>
+          <t xml:space="preserve">hsa-let-7b-3p</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7b-5p</t>
+          <t xml:space="preserve">mmu-let-7b-3p</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -1894,26 +1898,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6341898/</t>
-        </is>
-      </c>
+      <c r="E78"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">let-7b</t>
+          <t xml:space="preserve">let-7c</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7b-3p</t>
+          <t xml:space="preserve">hsa-let-7c-5p</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7b-3p</t>
+          <t xml:space="preserve">mmu-let-7c-5p</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -1921,7 +1921,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E79"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3256915/</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1931,12 +1935,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-let-7c-5p</t>
+          <t xml:space="preserve">hsa-let-7c-3p</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7c-5p</t>
+          <t xml:space="preserve">mmu-let-7c-1-3p</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -1944,11 +1948,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3256915/</t>
-        </is>
-      </c>
+      <c r="E80"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1956,14 +1956,10 @@
           <t xml:space="preserve">let-7c</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hsa-let-7c-3p</t>
-        </is>
-      </c>
+      <c r="B81"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7c-1-3p</t>
+          <t xml:space="preserve">mmu-let-7c-2-3p</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -1976,13 +1972,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">let-7c</t>
-        </is>
-      </c>
-      <c r="B82"/>
+          <t xml:space="preserve">miR-200a</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hsa-miR-200a-3p</t>
+        </is>
+      </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-let-7c-2-3p</t>
+          <t xml:space="preserve">mmu-miR-200a-3p</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -1990,7 +1990,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E82"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6307448/</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2000,12 +2004,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200a-3p</t>
+          <t xml:space="preserve">hsa-miR-200a-5p</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200a-3p</t>
+          <t xml:space="preserve">mmu-miR-200a-5p</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2013,26 +2017,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6307448/</t>
-        </is>
-      </c>
+      <c r="E83"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-200a</t>
+          <t xml:space="preserve">miR-200b</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200a-5p</t>
+          <t xml:space="preserve">hsa-miR-200b-3p</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200a-5p</t>
+          <t xml:space="preserve">mmu-miR-200b-3p</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2040,7 +2040,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E84"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.thelancet.com/article/S2352-3964(19)30349-4/fulltext</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2050,12 +2054,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200b-3p</t>
+          <t xml:space="preserve">hsa-miR-200b-5p</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200b-3p</t>
+          <t xml:space="preserve">mmu-miR-200b-5p</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2063,26 +2067,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.thelancet.com/article/S2352-3964(19)30349-4/fulltext</t>
-        </is>
-      </c>
+      <c r="E85"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-200b</t>
+          <t xml:space="preserve">miR-200c</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200b-5p</t>
+          <t xml:space="preserve">hsa-miR-200c-3p</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200b-5p</t>
+          <t xml:space="preserve">mmu-miR-200c-3p</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2090,7 +2090,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E86"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC10003123/</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2100,12 +2104,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200c-3p</t>
+          <t xml:space="preserve">hsa-miR-200c-5p</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200c-3p</t>
+          <t xml:space="preserve">mmu-miR-200c-5p</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2113,26 +2117,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC10003123/</t>
-        </is>
-      </c>
+      <c r="E87"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-200c</t>
+          <t xml:space="preserve">miR-205</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-200c-5p</t>
+          <t xml:space="preserve">hsa-miR-205-3p</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-200c-5p</t>
+          <t xml:space="preserve">mmu-miR-205-3p</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2140,7 +2140,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E88"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3583473/</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2150,12 +2154,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-205-3p</t>
+          <t xml:space="preserve">hsa-miR-205-5p</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-205-3p</t>
+          <t xml:space="preserve">mmu-miR-205-5p</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2163,26 +2167,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3583473/</t>
-        </is>
-      </c>
+      <c r="E89"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-205</t>
+          <t xml:space="preserve">miR-29a</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-205-5p</t>
+          <t xml:space="preserve">hsa-miR-29a-3p</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-205-5p</t>
+          <t xml:space="preserve">mmu-miR-29a-3p</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2190,7 +2190,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E90"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5431235/</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2200,12 +2204,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29a-3p</t>
+          <t xml:space="preserve">hsa-miR-29a-5p</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29a-3p</t>
+          <t xml:space="preserve">mmu-miR-29a-5p</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2213,26 +2217,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5431235/</t>
-        </is>
-      </c>
+      <c r="E91"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-29a</t>
+          <t xml:space="preserve">miR-29b</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29a-5p</t>
+          <t xml:space="preserve">hsa-miR-29b-3p</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29a-5p</t>
+          <t xml:space="preserve">mmu-miR-29b-3p</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2240,7 +2240,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E92"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.nature.com/articles/cddis2014304</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2250,12 +2254,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29b-3p</t>
+          <t xml:space="preserve">hsa-miR-29b-1-5p</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29b-3p</t>
+          <t xml:space="preserve">mmu-miR-29b-1-5p</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2263,11 +2267,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.nature.com/articles/cddis2014304</t>
-        </is>
-      </c>
+      <c r="E93"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2277,12 +2277,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29b-1-5p</t>
+          <t xml:space="preserve">hsa-miR-29b-2-5p</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29b-1-5p</t>
+          <t xml:space="preserve">mmu-miR-29b-2-5p</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2295,17 +2295,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-29b</t>
+          <t xml:space="preserve">miR-29c</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29b-2-5p</t>
+          <t xml:space="preserve">hsa-miR-29c-3p</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29b-2-5p</t>
+          <t xml:space="preserve">mmu-miR-29c-3p</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2313,7 +2313,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E95"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5956756/</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2323,12 +2327,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29c-3p</t>
+          <t xml:space="preserve">hsa-miR-29c-5p</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29c-3p</t>
+          <t xml:space="preserve">mmu-miR-29c-5p</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2336,26 +2340,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5956756/</t>
-        </is>
-      </c>
+      <c r="E96"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-29c</t>
+          <t xml:space="preserve">miR-30a</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-29c-5p</t>
+          <t xml:space="preserve">hsa-miR-30a-5p</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-29c-5p</t>
+          <t xml:space="preserve">mmu-miR-30a-5p</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2363,7 +2363,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E97"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ascopubs.org/doi/10.1200/JCO.2018.36.4_suppl.84</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2373,12 +2377,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30a-5p</t>
+          <t xml:space="preserve">hsa-miR-30a-3p</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30a-5p</t>
+          <t xml:space="preserve">mmu-miR-30a-3p</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2386,26 +2390,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://ascopubs.org/doi/10.1200/JCO.2018.36.4_suppl.84</t>
-        </is>
-      </c>
+      <c r="E98"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-30a</t>
+          <t xml:space="preserve">miR-30b</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30a-3p</t>
+          <t xml:space="preserve">hsa-miR-30b-5p</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30a-3p</t>
+          <t xml:space="preserve">mmu-miR-30b-5p</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2413,7 +2413,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E99"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24293274/</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2423,12 +2427,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30b-5p</t>
+          <t xml:space="preserve">hsa-miR-30b-3p</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30b-5p</t>
+          <t xml:space="preserve">mmu-miR-30b-3p</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2436,26 +2440,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24293274/</t>
-        </is>
-      </c>
+      <c r="E100"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-30b</t>
+          <t xml:space="preserve">miR-30c</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30b-3p</t>
+          <t xml:space="preserve">hsa-miR-30c-5p</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30b-3p</t>
+          <t xml:space="preserve">mmu-miR-30c-5p</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2463,7 +2463,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E101"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9972042/</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2473,12 +2477,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30c-5p</t>
+          <t xml:space="preserve">hsa-miR-30c-2-3p</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30c-5p</t>
+          <t xml:space="preserve">mmu-miR-30c-1-3p</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2486,11 +2490,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9972042/</t>
-        </is>
-      </c>
+      <c r="E102"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2500,12 +2500,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30c-2-3p</t>
+          <t xml:space="preserve">hsa-miR-30c-1-3p</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30c-1-3p</t>
+          <t xml:space="preserve">mmu-miR-30c-2-3p</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2518,17 +2518,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-30c</t>
+          <t xml:space="preserve">miR-101</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-30c-1-3p</t>
+          <t xml:space="preserve">hsa-miR-101-3p</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-30c-2-3p</t>
+          <t xml:space="preserve">mmu-miR-101a-3p</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2536,7 +2536,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E104"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9739992/</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2546,12 +2550,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-101-3p</t>
+          <t xml:space="preserve">hsa-miR-101-5p</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-101a-3p</t>
+          <t xml:space="preserve">mmu-miR-101a-5p</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2559,11 +2563,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9739992/</t>
-        </is>
-      </c>
+      <c r="E105"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2573,12 +2573,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-101-5p</t>
+          <t xml:space="preserve">hsa-miR-101-2-5p</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-101a-5p</t>
+          <t xml:space="preserve">mmu-miR-101b-5p</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2591,17 +2591,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-101</t>
+          <t xml:space="preserve">miR-122</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-101-2-5p</t>
+          <t xml:space="preserve">hsa-miR-122-5p</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-101b-5p</t>
+          <t xml:space="preserve">mmu-miR-122-5p</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2609,7 +2609,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E107"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/19296470/</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2619,12 +2623,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-122-5p</t>
+          <t xml:space="preserve">hsa-miR-122-3p</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-122-5p</t>
+          <t xml:space="preserve">mmu-miR-122-3p</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2632,26 +2636,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/19296470/</t>
-        </is>
-      </c>
+      <c r="E108"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-122</t>
+          <t xml:space="preserve">miR-184</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-122-3p</t>
+          <t xml:space="preserve">hsa-miR-184</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-122-3p</t>
+          <t xml:space="preserve">mmu-miR-184-3p</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2659,7 +2659,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E109"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6876683/</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2674,7 +2678,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-184-3p</t>
+          <t xml:space="preserve">mmu-miR-184-5p</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2682,26 +2686,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6876683/</t>
-        </is>
-      </c>
+      <c r="E110"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-184</t>
+          <t xml:space="preserve">miR-137</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-184</t>
+          <t xml:space="preserve">hsa-miR-137-3p</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-184-5p</t>
+          <t xml:space="preserve">mmu-miR-137-3p</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2709,7 +2709,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E111"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4494958/</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2719,12 +2723,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-137-3p</t>
+          <t xml:space="preserve">hsa-miR-137-5p</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-137-3p</t>
+          <t xml:space="preserve">mmu-miR-137-5p</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2732,26 +2736,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4494958/</t>
-        </is>
-      </c>
+      <c r="E112"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-137</t>
+          <t xml:space="preserve">miR-146a</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-137-5p</t>
+          <t xml:space="preserve">hsa-miR-146a-5p</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-137-5p</t>
+          <t xml:space="preserve">mmu-miR-146a-5p</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2759,7 +2759,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E113"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11896294/</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2769,12 +2773,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-146a-5p</t>
+          <t xml:space="preserve">hsa-miR-146a-3p</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-146a-5p</t>
+          <t xml:space="preserve">mmu-miR-146a-3p</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2782,26 +2786,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11896294/</t>
-        </is>
-      </c>
+      <c r="E114"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-146a</t>
+          <t xml:space="preserve">miR-149</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-146a-3p</t>
+          <t xml:space="preserve">hsa-miR-149-5p</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-146a-3p</t>
+          <t xml:space="preserve">mmu-miR-149-5p</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -2809,7 +2809,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E115"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://aacrjournals.org/cancerres/article/74/18/5256/597341/miR149-Functions-as-a-Tumor-Suppressor-by</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2819,12 +2823,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-149-5p</t>
+          <t xml:space="preserve">hsa-miR-149-3p</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-149-5p</t>
+          <t xml:space="preserve">mmu-miR-149-3p</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -2832,26 +2836,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://aacrjournals.org/cancerres/article/74/18/5256/597341/miR149-Functions-as-a-Tumor-Suppressor-by</t>
-        </is>
-      </c>
+      <c r="E116"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-149</t>
+          <t xml:space="preserve">miR-193b</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-149-3p</t>
+          <t xml:space="preserve">hsa-miR-193b-3p</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-149-3p</t>
+          <t xml:space="preserve">mmu-miR-193b-3p</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -2859,7 +2859,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E117"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6403503/</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2869,12 +2873,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-193b-3p</t>
+          <t xml:space="preserve">hsa-miR-193b-5p</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-193b-3p</t>
+          <t xml:space="preserve">mmu-miR-193b-5p</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -2882,26 +2886,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6403503/</t>
-        </is>
-      </c>
+      <c r="E118"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-193b</t>
+          <t xml:space="preserve">miR-203</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-193b-5p</t>
+          <t xml:space="preserve">hsa-miR-203a-3p</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-193b-5p</t>
+          <t xml:space="preserve">mmu-miR-203a-3p</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -2909,7 +2909,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E119"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4725318/</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2919,12 +2923,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-203a-3p</t>
+          <t xml:space="preserve">hsa-miR-203a-5p</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-203a-3p</t>
+          <t xml:space="preserve">mmu-miR-203a-5p</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -2932,11 +2936,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4725318/</t>
-        </is>
-      </c>
+      <c r="E120"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2946,12 +2946,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-203a-5p</t>
+          <t xml:space="preserve">hsa-miR-203b-3p</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-203a-5p</t>
+          <t xml:space="preserve">mmu-miR-203b-3p</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-203b-3p</t>
+          <t xml:space="preserve">hsa-miR-203b-5p</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-203b-3p</t>
+          <t xml:space="preserve">mmu-miR-203b-5p</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -2987,17 +2987,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-203</t>
+          <t xml:space="preserve">miR-218</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-203b-5p</t>
+          <t xml:space="preserve">hsa-miR-218-5p</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-203b-5p</t>
+          <t xml:space="preserve">mmu-miR-218-5p</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3005,7 +3005,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E123"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6896272/</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3015,12 +3019,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-218-5p</t>
+          <t xml:space="preserve">hsa-miR-218-1-3p</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-218-5p</t>
+          <t xml:space="preserve">mmu-miR-218-1-3p</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3028,11 +3032,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6896272/</t>
-        </is>
-      </c>
+      <c r="E124"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-218-1-3p</t>
+          <t xml:space="preserve">hsa-miR-218-2-3p</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-218-1-3p</t>
+          <t xml:space="preserve">mmu-miR-218-2-3p</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3060,17 +3060,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-218</t>
+          <t xml:space="preserve">miR-223</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-218-2-3p</t>
+          <t xml:space="preserve">hsa-miR-223-3p</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-218-2-3p</t>
+          <t xml:space="preserve">mmu-miR-223-3p</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3078,7 +3078,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E126"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/33951281/</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3088,12 +3092,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-223-3p</t>
+          <t xml:space="preserve">hsa-miR-223-5p</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-223-3p</t>
+          <t xml:space="preserve">mmu-miR-223-5p</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3101,26 +3105,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/33951281/</t>
-        </is>
-      </c>
+      <c r="E127"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-223</t>
+          <t xml:space="preserve">miR-451</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-223-5p</t>
+          <t xml:space="preserve">hsa-miR-451a</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-223-5p</t>
+          <t xml:space="preserve">mmu-miR-451a</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3128,7 +3128,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E128"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/21358675/</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3138,12 +3142,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-451a</t>
+          <t xml:space="preserve">hsa-miR-451b</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-451a</t>
+          <t xml:space="preserve">mmu-miR-451b</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3151,34 +3155,30 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/21358675/</t>
-        </is>
-      </c>
+      <c r="E129"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-451</t>
+          <t xml:space="preserve">miR-506</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-451b</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mmu-miR-451b</t>
-        </is>
-      </c>
+          <t xml:space="preserve">hsa-miR-506-3p</t>
+        </is>
+      </c>
+      <c r="C130"/>
       <c r="D130" t="inlineStr">
         <is>
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E130"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24608427/</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-506-3p</t>
+          <t xml:space="preserve">hsa-miR-506-5p</t>
         </is>
       </c>
       <c r="C131"/>
@@ -3197,21 +3197,17 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/24608427/</t>
-        </is>
-      </c>
+      <c r="E131"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-506</t>
+          <t xml:space="preserve">miR-612</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-506-5p</t>
+          <t xml:space="preserve">hsa-miR-612</t>
         </is>
       </c>
       <c r="C132"/>
@@ -3220,20 +3216,28 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E132"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5919718/</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-612</t>
+          <t xml:space="preserve">miR-7</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-612</t>
-        </is>
-      </c>
-      <c r="C133"/>
+          <t xml:space="preserve">hsa-miR-7-5p</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mmu-miR-7a-5p</t>
+        </is>
+      </c>
       <c r="D133" t="inlineStr">
         <is>
           <t xml:space="preserve">Tumor suppressor</t>
@@ -3241,7 +3245,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5919718/</t>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5360436/</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3257,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-7-5p</t>
+          <t xml:space="preserve">hsa-miR-7-1-3p</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-7a-5p</t>
+          <t xml:space="preserve">mmu-miR-7b-5p</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -3266,11 +3270,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC5360436/</t>
-        </is>
-      </c>
+      <c r="E134"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3280,12 +3280,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-7-1-3p</t>
+          <t xml:space="preserve">hsa-miR-7-2-3p</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-7b-5p</t>
+          <t xml:space="preserve">mmu-miR-7a-1-3p</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -3301,14 +3301,10 @@
           <t xml:space="preserve">miR-7</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hsa-miR-7-2-3p</t>
-        </is>
-      </c>
+      <c r="B136"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-7a-1-3p</t>
+          <t xml:space="preserve">mmu-miR-7a-2-3p</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -3327,7 +3323,7 @@
       <c r="B137"/>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-7a-2-3p</t>
+          <t xml:space="preserve">mmu-miR-7b-3p</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -3340,13 +3336,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-7</t>
-        </is>
-      </c>
-      <c r="B138"/>
+          <t xml:space="preserve">miR-9</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hsa-miR-9-5p</t>
+        </is>
+      </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-7b-3p</t>
+          <t xml:space="preserve">mmu-miR-9-5p</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -3354,7 +3354,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E138"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6614627/</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3364,12 +3368,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-9-5p</t>
+          <t xml:space="preserve">hsa-miR-9-3p</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-9-5p</t>
+          <t xml:space="preserve">mmu-miR-9-3p</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -3377,26 +3381,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6614627/</t>
-        </is>
-      </c>
+      <c r="E139"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-9</t>
+          <t xml:space="preserve">miR-100</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-9-3p</t>
+          <t xml:space="preserve">hsa-miR-100-5p</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-9-3p</t>
+          <t xml:space="preserve">mmu-miR-100-5p</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -3404,7 +3404,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E140"/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11875724/</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3414,12 +3418,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-100-5p</t>
+          <t xml:space="preserve">hsa-miR-100-3p</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-100-5p</t>
+          <t xml:space="preserve">mmu-miR-100-3p</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -3427,26 +3431,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11875724/</t>
-        </is>
-      </c>
+      <c r="E141"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-100</t>
+          <t xml:space="preserve">miR-181a</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-100-3p</t>
+          <t xml:space="preserve">hsa-miR-181a-5p</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-100-3p</t>
+          <t xml:space="preserve">mmu-miR-181a-5p</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3454,7 +3454,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E142"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC10725356/</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3464,12 +3468,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181a-5p</t>
+          <t xml:space="preserve">hsa-miR-181a-3p</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181a-5p</t>
+          <t xml:space="preserve">mmu-miR-181a-1-3p</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3477,11 +3481,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC10725356/</t>
-        </is>
-      </c>
+      <c r="E143"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3491,12 +3491,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181a-3p</t>
+          <t xml:space="preserve">hsa-miR-181a-2-3p</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181a-1-3p</t>
+          <t xml:space="preserve">mmu-miR-181a-2-3p</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -3509,17 +3509,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-181a</t>
+          <t xml:space="preserve">miR-181b</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181a-2-3p</t>
+          <t xml:space="preserve">hsa-miR-181b-5p</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181a-2-3p</t>
+          <t xml:space="preserve">mmu-miR-181b-5p</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3527,7 +3527,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E145"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3596691/</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3537,12 +3541,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181b-5p</t>
+          <t xml:space="preserve">hsa-miR-181b-3p</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181b-5p</t>
+          <t xml:space="preserve">mmu-miR-181b-1-3p</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -3550,11 +3554,7 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC3596691/</t>
-        </is>
-      </c>
+      <c r="E146"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3564,12 +3564,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181b-3p</t>
+          <t xml:space="preserve">hsa-miR-181b-2-3p</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181b-1-3p</t>
+          <t xml:space="preserve">mmu-miR-181b-2-3p</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -3582,17 +3582,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-181b</t>
+          <t xml:space="preserve">miR-215</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-181b-2-3p</t>
+          <t xml:space="preserve">hsa-miR-215-5p</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-181b-2-3p</t>
+          <t xml:space="preserve">mmu-miR-215-5p</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -3600,7 +3600,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E148"/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4579799/</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3610,12 +3614,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-215-5p</t>
+          <t xml:space="preserve">hsa-miR-215-3p</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-215-5p</t>
+          <t xml:space="preserve">mmu-miR-215-3p</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3623,26 +3627,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4579799/</t>
-        </is>
-      </c>
+      <c r="E149"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-215</t>
+          <t xml:space="preserve">miR-195</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-215-3p</t>
+          <t xml:space="preserve">hsa-miR-195-5p</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-215-3p</t>
+          <t xml:space="preserve">mmu-miR-195a-5p</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3650,7 +3650,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E150"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3660,12 +3664,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-195-5p</t>
+          <t xml:space="preserve">hsa-miR-195-3p</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-195a-5p</t>
+          <t xml:space="preserve">mmu-miR-195a-3p</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3673,26 +3677,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
-        </is>
-      </c>
+      <c r="E151"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-195</t>
+          <t xml:space="preserve">miR-216a</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-195-3p</t>
+          <t xml:space="preserve">hsa-miR-216a-5p</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-195a-3p</t>
+          <t xml:space="preserve">mmu-miR-216a-5p</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3700,7 +3700,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E152"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9899407/</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3710,12 +3714,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-216a-5p</t>
+          <t xml:space="preserve">hsa-miR-216a-3p</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-216a-5p</t>
+          <t xml:space="preserve">mmu-miR-216a-3p</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -3723,26 +3727,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC9899407/</t>
-        </is>
-      </c>
+      <c r="E153"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-216a</t>
+          <t xml:space="preserve">miR-320a</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-216a-3p</t>
+          <t xml:space="preserve">hsa-miR-320a-3p</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-216a-3p</t>
+          <t xml:space="preserve">mmu-miR-320-3p</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3750,7 +3750,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E154"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/33833996/</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3760,12 +3764,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-320a-3p</t>
+          <t xml:space="preserve">hsa-miR-320a-5p</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-320-3p</t>
+          <t xml:space="preserve">mmu-miR-320-5p</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3773,26 +3777,22 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/33833996/</t>
-        </is>
-      </c>
+      <c r="E155"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">miR-320a</t>
+          <t xml:space="preserve">miR-199a</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-320a-5p</t>
+          <t xml:space="preserve">hsa-miR-199a-5p</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-320-5p</t>
+          <t xml:space="preserve">mmu-miR-199a-5p</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3800,7 +3800,11 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E156"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3810,12 +3814,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">hsa-miR-199a-5p</t>
+          <t xml:space="preserve">hsa-miR-199a-3p</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">mmu-miR-199a-5p</t>
+          <t xml:space="preserve">mmu-miR-199a-3p</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3823,36 +3827,9 @@
           <t xml:space="preserve">Tumor suppressor</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC4943968/</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">miR-199a</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hsa-miR-199a-3p</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mmu-miR-199a-3p</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tumor suppressor</t>
-        </is>
-      </c>
-      <c r="E158"/>
+      <c r="E157"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E158"/>
+  <autoFilter ref="A1:E157"/>
 </worksheet>
 </file>
</xml_diff>